<commit_message>
Phase 1.1: Updated indexed data sheet
</commit_message>
<xml_diff>
--- a/docs/PonniRAG –  Indexed Data.xlsx
+++ b/docs/PonniRAG –  Indexed Data.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="31">
   <si>
     <t>Volume</t>
   </si>
@@ -34,7 +34,7 @@
     <t>Vol 1</t>
   </si>
   <si>
-    <t>8(Issues 6–12 + Pongal Issue)</t>
+    <t>8(Issues 6-12 + Pongal Issue)</t>
   </si>
   <si>
     <t>Issues 6, 7, 8, 9, 10, 11, 12, Pongal Issue</t>
@@ -46,7 +46,7 @@
     <t>Vol 2</t>
   </si>
   <si>
-    <t>18(Issues 1–18)</t>
+    <t>18(Issues 1-18)</t>
   </si>
   <si>
     <t>Issues 1–18</t>
@@ -55,43 +55,37 @@
     <t>Vol 3</t>
   </si>
   <si>
-    <t>23(Issues 1–23)</t>
+    <t>23(Issues 1-23)</t>
   </si>
   <si>
-    <t>Issues 1–19, 21–23</t>
-  </si>
-  <si>
-    <t>Issue 20 (Proofread document not available earlier)</t>
+    <t>Issues 1–23</t>
   </si>
   <si>
     <t>Vol 4</t>
   </si>
   <si>
-    <t>11(Issues 1–11)</t>
+    <t>11(Issues 1-11)</t>
   </si>
   <si>
-    <t>Issues 1, 4, 5, 7</t>
-  </si>
-  <si>
-    <t>Issues 6, 8, 9, 10, 11 (Proofread documents not yet provided)</t>
+    <t>Issues 1, 4-11</t>
   </si>
   <si>
     <t>Vol 5</t>
   </si>
   <si>
-    <t>21(Issues 1–21)</t>
+    <t>21(Issues 1-21)</t>
   </si>
   <si>
-    <t>Issues 1–21</t>
+    <t>Issues 1-21</t>
   </si>
   <si>
     <t>Vol 6</t>
   </si>
   <si>
-    <t>22(Issues 1–21 + Pongal Issue)</t>
+    <t>18(Issues 1-12,14,17,19-21 + Pongal Issue)</t>
   </si>
   <si>
-    <t>Issues 1, 2 (named as Issue 3), 3, 4, 5, 6, 7, 9–14, 19–21, Pongal Issue (Proofread available but not indexed)</t>
+    <t>Issues 1-12,14,17,19-21 + Pongal Issue)</t>
   </si>
   <si>
     <t>Vol 7</t>
@@ -100,23 +94,23 @@
     <t>1 issue</t>
   </si>
   <si>
-    <t>All issues (No proofread documents provided)</t>
-  </si>
-  <si>
     <t>Vol 8</t>
   </si>
   <si>
-    <t>12(Issues 1-12)</t>
+    <t>10(Issues 1-4,6-8,10-12)</t>
   </si>
   <si>
-    <t>Issues 6, 7, 12 (Proofread available but not indexed)</t>
+    <t>Issues 1-4,6-8,10-12</t>
+  </si>
+  <si>
+    <t>Total Issues</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -138,6 +132,11 @@
       <color theme="1"/>
       <name val="Arial"/>
     </font>
+    <font>
+      <b/>
+      <color theme="1"/>
+      <name val="Arial"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -147,24 +146,44 @@
       <patternFill patternType="lightGray"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border/>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="1" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -524,13 +543,13 @@
         <v>15</v>
       </c>
       <c r="D4" s="3">
-        <v>22.0</v>
+        <v>23.0</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="F4" s="3">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="G4" s="2"/>
       <c r="H4" s="2"/>
@@ -556,22 +575,22 @@
     </row>
     <row r="5">
       <c r="A5" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="C5" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="C5" s="3" t="s">
-        <v>19</v>
-      </c>
       <c r="D5" s="3">
-        <v>4.0</v>
+        <v>9.0</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="F5" s="3">
-        <v>5.0</v>
+        <v>0.0</v>
       </c>
       <c r="G5" s="2"/>
       <c r="H5" s="2"/>
@@ -597,13 +616,13 @@
     </row>
     <row r="6">
       <c r="A6" s="3" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D6" s="3">
         <v>21.0</v>
@@ -638,22 +657,22 @@
     </row>
     <row r="7">
       <c r="A7" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C7" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B7" s="3" t="s">
-        <v>25</v>
+      <c r="D7" s="3">
+        <v>18.0</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="E7" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D7" s="3">
+      <c r="F7" s="3">
         <v>0.0</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="F7" s="3">
-        <v>21.0</v>
       </c>
       <c r="G7" s="2"/>
       <c r="H7" s="2"/>
@@ -679,22 +698,22 @@
     </row>
     <row r="8">
       <c r="A8" s="3" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="D8" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="E8" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D8" s="3">
+      <c r="F8" s="3">
         <v>0.0</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="F8" s="3">
-        <v>1.0</v>
       </c>
       <c r="G8" s="2"/>
       <c r="H8" s="2"/>
@@ -720,22 +739,22 @@
     </row>
     <row r="9">
       <c r="A9" s="3" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C9" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D9" s="3">
+        <v>10.0</v>
+      </c>
+      <c r="E9" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D9" s="3">
+      <c r="F9" s="3">
         <v>0.0</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="F9" s="3">
-        <v>12.0</v>
       </c>
       <c r="G9" s="2"/>
       <c r="H9" s="2"/>
@@ -762,8 +781,13 @@
     <row r="10">
       <c r="A10" s="2"/>
       <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
+      <c r="C10" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="D10" s="5">
+        <f>SUM(D2:D9)</f>
+        <v>108</v>
+      </c>
       <c r="E10" s="2"/>
       <c r="F10" s="2"/>
       <c r="G10" s="2"/>

</xml_diff>